<commit_message>
🔄 更新看板 08/12 14:50
</commit_message>
<xml_diff>
--- a/导出_线下个案.xlsx
+++ b/导出_线下个案.xlsx
@@ -802,7 +802,7 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>100000</v>
+        <v>50000</v>
       </c>
       <c r="D8" t="n">
         <v>0</v>
@@ -854,14 +854,14 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>280000</v>
+        <v>150000</v>
       </c>
       <c r="D9" t="n">
         <v>12116.3</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>4.3%</t>
+          <t>8.1%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -906,14 +906,14 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>50000</v>
+        <v>130000</v>
       </c>
       <c r="D10" t="n">
         <v>16196</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>32.4%</t>
+          <t>12.5%</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -958,14 +958,14 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>73000</v>
+        <v>160000</v>
       </c>
       <c r="D11" t="n">
         <v>29798</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>40.8%</t>
+          <t>18.6%</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -1006,47 +1006,47 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>李明</t>
+          <t>钟燕红</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>120000</v>
+        <v>270000</v>
       </c>
       <c r="D12" t="n">
-        <v>53484</v>
+        <v>103420.75</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>44.6%</t>
+          <t>38.3%</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>+142.0%</t>
+          <t>+50.8%</t>
         </is>
       </c>
       <c r="G12" t="n">
-        <v>7000</v>
+        <v>15580</v>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>13.1%</t>
+          <t>15.1%</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>+133.3%</t>
+          <t>-24.1%</t>
         </is>
       </c>
       <c r="J12" t="n">
-        <v>46484</v>
+        <v>87840.75</v>
       </c>
       <c r="K12" t="n">
-        <v>19098</v>
+        <v>46452</v>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>+143.4%</t>
+          <t>+89.1%</t>
         </is>
       </c>
     </row>
@@ -1058,47 +1058,47 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>钟燕红</t>
+          <t>李明</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>100000</v>
+        <v>120000</v>
       </c>
       <c r="D13" t="n">
-        <v>103420.75</v>
+        <v>53484</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>103.4%</t>
+          <t>44.6%</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>+50.8%</t>
+          <t>+142.0%</t>
         </is>
       </c>
       <c r="G13" t="n">
-        <v>15580</v>
+        <v>7000</v>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>15.1%</t>
+          <t>13.1%</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>-24.1%</t>
+          <t>+133.3%</t>
         </is>
       </c>
       <c r="J13" t="n">
-        <v>87840.75</v>
+        <v>46484</v>
       </c>
       <c r="K13" t="n">
-        <v>46452</v>
+        <v>19098</v>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>+89.1%</t>
+          <t>+143.4%</t>
         </is>
       </c>
     </row>

</xml_diff>